<commit_message>
Update preliminary submission pack: revised tech report exports, offline verification, and code package.
Sync review fixes into the report Markdown/DOCX/PDF pipeline, refresh designated-set offline materials, and repack the XH-202610 source bundle for GitHub backup.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/资料/初赛材料/02_离线验证/交稿/离线性能验证报告_XH-202610.xlsx
+++ b/资料/初赛材料/02_离线验证/交稿/离线性能验证报告_XH-202610.xlsx
@@ -215,7 +215,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>11</row>
+      <row>14</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6096000" cy="3619500"/>
@@ -240,7 +240,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>31</row>
+      <row>34</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6096000" cy="3629025"/>
@@ -265,7 +265,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>51</row>
+      <row>54</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6096000" cy="4819650"/>
@@ -290,7 +290,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>71</row>
+      <row>74</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6096000" cy="3629025"/>
@@ -613,7 +613,7 @@
     <col width="23.2" customWidth="1" min="5" max="5"/>
     <col width="35.2" customWidth="1" min="6" max="6"/>
     <col width="21.4" customWidth="1" min="7" max="7"/>
-    <col width="28.4" customWidth="1" min="8" max="8"/>
+    <col width="35.2" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
@@ -699,7 +699,7 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>原始/nested_N0_metrics.json</t>
+          <t>原始验证数据/nested_N0_metrics.json</t>
         </is>
       </c>
     </row>
@@ -858,7 +858,7 @@
     <row r="13" ht="22" customHeight="1">
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>测试集 S07/S08 共 120 trial、无标签：盲测预测见 原始/submission_QuadFold59.csv；未使用测试标签调参，故准/召/特以 train 嵌套主读为准。</t>
+          <t>测试集 S07/S08 共 120 trial、无标签：盲测预测已写入官方模板 原始验证数据/sample_submission.csv；未使用测试标签调参，故准/召/特以 train 嵌套主读为准。</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
     <row r="16" ht="22" customHeight="1">
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>来源：Exp37 nested-S0（N0）OOF 概率 argmax；文件 原始/nested_N0_metrics.json 与 原始/oof_N0/。</t>
+          <t>来源：Exp37 nested-S0（N0）OOF 概率 argmax；文件 原始验证数据/nested_N0_metrics.json 与 原始验证数据/oof_N0/。</t>
         </is>
       </c>
     </row>
@@ -1497,7 +1497,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="67.80000000000004" customWidth="1" min="2" max="2"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
     <col width="70.60000000000002" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -1663,7 +1663,7 @@
     <row r="17" ht="22" customHeight="1">
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>完整文字版见交稿包：数据集使用说明.md；官方原文副本见 原始/官方数据说明.md。</t>
+          <t>完整文字版见交稿包：数据集使用说明.md；官方原文副本见 原始验证数据/官方数据说明.md。</t>
         </is>
       </c>
     </row>
@@ -1687,7 +1687,7 @@
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="56" customWidth="1" min="2" max="2"/>
     <col width="39.40000000000001" customWidth="1" min="3" max="3"/>
-    <col width="35.3" customWidth="1" min="4" max="4"/>
+    <col width="38.2" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -1730,7 +1730,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>原始/nested_N0_metrics.json</t>
+          <t>原始验证数据/nested_N0_metrics.json</t>
         </is>
       </c>
     </row>
@@ -1742,16 +1742,16 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>盲测交卷预测 CSV（120 行）</t>
+          <t>盲测交卷预测 CSV（官方模板已填 label）</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>原始/submission_QuadFold59.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
+          <t>原始验证数据/sample_submission.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="38" customHeight="1">
       <c r="B7" s="4" t="inlineStr">
         <is>
           <t>D3</t>
@@ -1759,12 +1759,12 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>官方提交模板（行序对照）</t>
+          <t>同内容内部备份（模型名归档）</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>原始/sample_submission.csv</t>
+          <t>原始验证数据/submission_QuadFold59.csv</t>
         </is>
       </c>
     </row>
@@ -1781,7 +1781,7 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>原始/oof_N0/oof_N0_*.npy</t>
+          <t>原始验证数据/oof_N0/oof_N0_*.npy</t>
         </is>
       </c>
     </row>
@@ -1798,7 +1798,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>原始/官方数据说明.md</t>
+          <t>原始验证数据/官方数据说明.md</t>
         </is>
       </c>
     </row>
@@ -1815,7 +1815,7 @@
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>原始/数据说明_使用对照.md</t>
+          <t>原始验证数据/数据说明_使用对照.md</t>
         </is>
       </c>
     </row>
@@ -1832,11 +1832,11 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>截图/</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="38" customHeight="1">
+          <t>验证过程截图/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
       <c r="B12" s="6" t="inlineStr">
         <is>
           <t>D8</t>
@@ -1875,13 +1875,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:F10"/>
+  <dimension ref="A2:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="43.1" customWidth="1" min="2" max="2"/>
-    <col width="30.49999999999999" customWidth="1" min="3" max="3"/>
-    <col width="33" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="38.2" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
   </cols>
@@ -1925,12 +1925,12 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>指定集目录与 PKL 结构核验</t>
+          <t>指定集官方数据核验：目录树、PKL 结构（data 64×22500、ch_names、srate=250）、train 900 / test 120 计数（终端回放）</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>截图/S01_指定集目录与pkl结构.png</t>
+          <t>验证过程截图/S01_数据集结构与加载核验.png</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -1947,12 +1947,12 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>嵌套 N0 主读 Acc/召/特/F1 汇总</t>
+          <t>嵌套 N0 主读回放运行：replay_nested.py 现场输出六折 Acc 与 0.511±0.066（终端回放）</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>截图/S02_嵌套N0指标汇总.png</t>
+          <t>验证过程截图/S02_嵌套N0指标汇总.png</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -1969,12 +1969,12 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>交卷 CSV 前 30 行与标签分布</t>
+          <t>盲测交卷 CSV 再生成与比对：predict_submission.py 现场重生成，与交稿 CSV 逐行 diff（终端回放）</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>截图/S03_交卷CSV前30行.png</t>
+          <t>验证过程截图/S03_交卷CSV再生成与比对.png</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -1991,12 +1991,12 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>核心指标填写说明（准/召/特/延迟）</t>
+          <t>指定集指标独立复算：从 OOF npy 重算 Acc/召/特/F1/CM/六折，逐项对照登记 JSON（终端回放）</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>截图/S04_Excel总表指定集行说明.png</t>
+          <t>验证过程截图/S04_独立复算.png</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -2005,11 +2005,77 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
-    <row r="10">
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>下列嵌入图便于审阅；原图亦在交稿/验证过程截图/。</t>
+    <row r="9" ht="22" customHeight="1">
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>交卷 CSV 完整性：120 行、表头一致、sample_id 与官方模板逐行对齐、取值合法（终端回放）</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>验证过程截图/S05_交卷CSV完整性校验.png</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>S06</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Excel 核心指标与登记 JSON 一致性：程序化读取 00 表单元格对照（终端回放）</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>验证过程截图/S06_Excel与JSON一致性.png</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>S07</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>交稿包文件 MD5 指纹与运行环境（python/numpy 版本、时间戳；终端回放）</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>验证过程截图/S07_文件指纹与环境.png</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>下列嵌入图便于审阅；原图亦在交稿包 验证过程截图/ 目录。</t>
         </is>
       </c>
     </row>
@@ -2092,7 +2158,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>submission_QuadFold59.csv（120 行，label∈{0,1,2}）</t>
+          <t>sample_submission.csv（官方模板已填 label∈{0,1,2}，120 行）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync preliminary materials and report assets with latest offline pack and figures.
Include revised tech report drafts/figures, offline verification pack updates, code package refresh, and Leave-Next tooling; keep submission numbers unchanged.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/资料/初赛材料/02_离线验证/交稿/离线性能验证报告_XH-202610.xlsx
+++ b/资料/初赛材料/02_离线验证/交稿/离线性能验证报告_XH-202610.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="22320" windowHeight="11480" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_核心指标" sheetId="1" state="visible" r:id="rId1"/>
@@ -18,7 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_数据核对" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -27,41 +26,197 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="26">
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <name val="宋体"/>
+      <charset val="134"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
       <name val="Noto Sans SC"/>
-      <color rgb="001B2A4A"/>
+      <charset val="134"/>
+      <color rgb="FF1B2A4A"/>
       <sz val="16"/>
     </font>
     <font>
       <name val="Noto Sans SC"/>
-      <color rgb="008C8A84"/>
+      <charset val="134"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Noto Sans SC"/>
+      <charset val="134"/>
+      <color rgb="FF37352F"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Noto Sans SC"/>
+      <charset val="134"/>
+      <color rgb="FF8C8A84"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Noto Sans SC"/>
-      <color rgb="00FFFFFF"/>
+      <charset val="134"/>
+      <color rgb="FF1B2A4A"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Noto Sans SC"/>
-      <color rgb="0037352F"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <color theme="1"/>
       <sz val="11"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <name val="Noto Sans SC"/>
-      <color rgb="001B2A4A"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF0000FF"/>
       <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="15"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="13"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF3F3F76"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FF3F3F3F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF006100"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF9C0006"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF9C6500"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color theme="0"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="36">
     <fill>
       <patternFill/>
     </fill>
@@ -70,21 +225,210 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001B2A4A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F7F7F5"/>
+        <fgColor rgb="FF1B2A4A"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF7F7F5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -93,49 +437,358 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="thin">
-        <color rgb="00E9E9E8"/>
+        <color rgb="FFE9E9E8"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="49">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="34" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="35" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="49">
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -218,7 +871,7 @@
       <row>14</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6096000" cy="3619500"/>
+    <ext cx="8572500" cy="3190875"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -240,10 +893,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>34</row>
+      <row>33</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6096000" cy="3629025"/>
+    <ext cx="8572500" cy="4219575"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -265,10 +918,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>54</row>
+      <row>58</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6096000" cy="4819650"/>
+    <ext cx="8572500" cy="2333625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="3" name="Image 3" descr="Picture"/>
@@ -290,10 +943,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>74</row>
+      <row>73</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6096000" cy="3629025"/>
+    <ext cx="8572500" cy="2943225"/>
     <pic>
       <nvPicPr>
         <cNvPr id="4" name="Image 4" descr="Picture"/>
@@ -301,6 +954,81 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>91</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="1885950"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>103</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="2009775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>116</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="3476625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -593,7 +1321,6 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -603,8 +1330,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B2:H14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
@@ -625,223 +1352,223 @@
       </c>
     </row>
     <row r="3" ht="8" customHeight="1">
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>本报告仅报告主办方指定标准脑电数据集（Challenge MI / S01–S08）上的算法性能；不含自采数据与其他公开库读数。</t>
         </is>
       </c>
     </row>
     <row r="5" ht="28" customHeight="1">
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>指标（官方要求）</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>数值</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>口径说明</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>模型</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>评测协议</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>评测方案</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>样本规模</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>证据文件</t>
         </is>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1">
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>分类准确率</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="14" t="n">
         <v>0.5111</v>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>三分类试次级 Acc；类均衡下与 macro 召回同值</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>QuadFold-59</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>LOSO6 · leave-fold 嵌套 Val（主读）</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>900 trial（S01–S06）</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>留一被试交叉验证 6 折（LOSO6）· 嵌套验证集（主要结果）</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>900 试次（S01–S06）</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>原始验证数据/nested_N0_metrics.json</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>召回率（macro）</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="15" t="n">
         <v>0.5111</v>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>三类召回率算术平均</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>QuadFold-59</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>同上</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>每类 300 trial</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>每类 300 试次</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>同上</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>特异性（macro）</t>
         </is>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" s="14" t="n">
         <v>0.7556</v>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>三类特异性算术平均</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>QuadFold-59</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>同上</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>同上</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>同上</t>
         </is>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1">
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>运算延迟（单 trial 前向）</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>运算延迟（单试次前向）</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>1.11 ms</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>RTX 5070；3 s / 750 点窗；四成员融合链路单窗增量</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>QuadFold-59（同构推理）</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>离线批推理计时</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>单窗</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>sheet 03</t>
         </is>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1">
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>判定延迟（协议上界）</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>判定延迟（实验范式时序上界）</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>3.00 s</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>指定集 1 trial = 1 窗（750 点）；无滑窗 hop；+前向 1.11 ms</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>指定集 1 试次 = 1 窗（750 点）；无滑窗步长；+前向 1.11 ms</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>QuadFold-59</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>官方 trial 切分</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>单 trial</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>官方试次切分</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>单试次</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>sheet 03 · 官方数据说明</t>
         </is>
@@ -849,23 +1576,23 @@
     </row>
     <row r="11" ht="22" customHeight="1"/>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>附报（不作主读）：折内 Val Acc=0.558±0.069（融合参数本折拟合，乐观偏置约 +4.7 pp）。</t>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>附报（不作主要结果）：折内验证准确率 0.5580 ± 0.0690（融合参数在本折内拟合，存在约 4.7 个百分点的乐观偏置）。</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>测试集 S07/S08 共 120 trial、无标签：盲测预测已写入官方模板 原始验证数据/sample_submission.csv；未使用测试标签调参，故准/召/特以 train 嵌套主读为准。</t>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>测试集 S07/S08 共 120 试次、无标签：盲测预测已写入官方模板 原始验证数据/sample_submission.csv；未使用测试标签调参，故准确率/召回率/特异性以训练集嵌套验证的主要结果为准。</t>
         </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>交卷模型：QuadFold-59 = 59 EEG 通道、从零训练的四成员温度校准集成（内部代号 S0 / E1f-A59）。</t>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>提交模型：QuadFold-59 = 59 通道脑电、从零训练的四成员温度校准集成。</t>
         </is>
       </c>
     </row>
@@ -883,17 +1610,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B2:H16"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="3" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
@@ -906,39 +1628,39 @@
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="28" customHeight="1">
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>类别</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>支持数</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>召回率</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>特异性</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>精确率</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>F1</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>左手运动想象 / Left(0)</t>
         </is>
@@ -946,43 +1668,43 @@
       <c r="C5" s="8" t="n">
         <v>300</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" s="14" t="n">
         <v>0.3267</v>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="E5" s="14" t="n">
         <v>0.85</v>
       </c>
-      <c r="F5" s="5" t="n">
+      <c r="F5" s="14" t="n">
         <v>0.5213</v>
       </c>
-      <c r="G5" s="5" t="n">
+      <c r="G5" s="14" t="n">
         <v>0.4016</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>右手运动想象 / Right(1)</t>
         </is>
       </c>
-      <c r="C6" s="9" t="n">
+      <c r="C6" s="7" t="n">
         <v>300</v>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="15" t="n">
         <v>0.6233</v>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="E6" s="15" t="n">
         <v>0.7117</v>
       </c>
-      <c r="F6" s="7" t="n">
+      <c r="F6" s="15" t="n">
         <v>0.5194</v>
       </c>
-      <c r="G6" s="7" t="n">
+      <c r="G6" s="15" t="n">
         <v>0.5667</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>静息态（空闲） / Rest(2)</t>
         </is>
@@ -990,69 +1712,69 @@
       <c r="C7" s="8" t="n">
         <v>300</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="14" t="n">
         <v>0.5833</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="14" t="n">
         <v>0.705</v>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="F7" s="14" t="n">
         <v>0.4972</v>
       </c>
-      <c r="G7" s="5" t="n">
+      <c r="G7" s="14" t="n">
         <v>0.5368000000000001</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>macro / 总体</t>
         </is>
       </c>
-      <c r="C8" s="9" t="n">
+      <c r="C8" s="7" t="n">
         <v>900</v>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="D8" s="15" t="n">
         <v>0.5111</v>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="E8" s="15" t="n">
         <v>0.7556</v>
       </c>
-      <c r="F8" s="7" t="n">
+      <c r="F8" s="15" t="n">
         <v>0.5125999999999999</v>
       </c>
-      <c r="G8" s="7" t="n">
+      <c r="G8" s="15" t="n">
         <v>0.5017</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1"/>
     <row r="10" ht="24" customHeight="1">
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>混淆矩阵（行=真实，列=预测；类序 左 / 右 / 静息）</t>
         </is>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
-      <c r="B11" s="3" t="inlineStr"/>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr"/>
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>预测·左手</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>预测·右手</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>预测·静息</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>真实·左手</t>
         </is>
@@ -1068,23 +1790,23 @@
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>真实·右手</t>
         </is>
       </c>
-      <c r="C13" s="9" t="n">
+      <c r="C13" s="7" t="n">
         <v>46</v>
       </c>
-      <c r="D13" s="9" t="n">
+      <c r="D13" s="7" t="n">
         <v>187</v>
       </c>
-      <c r="E13" s="9" t="n">
+      <c r="E13" s="7" t="n">
         <v>67</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>真实·静息</t>
         </is>
@@ -1101,9 +1823,9 @@
     </row>
     <row r="15" ht="22" customHeight="1"/>
     <row r="16" ht="22" customHeight="1">
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>来源：Exp37 nested-S0（N0）OOF 概率 argmax；文件 原始验证数据/nested_N0_metrics.json 与 原始验证数据/oof_N0/。</t>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>来源：嵌套验证折外预测（OOF）概率逐试次取最大类别；文件 原始验证数据/nested_N0_metrics.json 与 原始验证数据/oof_N0/。</t>
         </is>
       </c>
     </row>
@@ -1122,17 +1844,18 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="3" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="29.09999999999999" customWidth="1" min="6" max="6"/>
+    <col width="29.1" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1"/>
+    <row r="1" ht="15" customHeight="1">
+      <c r="A1" s="10" t="n"/>
+    </row>
     <row r="2" ht="32" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -1142,37 +1865,37 @@
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="38" customHeight="1">
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>折</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>保留被试（Val）</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Val 试次数</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>嵌套 Acc</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>说明</t>
         </is>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1">
-      <c r="B5" s="8" t="n">
+      <c r="B5" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>S01</t>
         </is>
@@ -1180,41 +1903,41 @@
       <c r="D5" s="8" t="n">
         <v>150</v>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="E5" s="14" t="n">
         <v>0.4267</v>
       </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>融合参数仅在其余五折 OOF 上拟合</t>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>融合参数仅在其余五折的折外预测（OOF）上拟合</t>
         </is>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1">
-      <c r="B6" s="9" t="n">
+      <c r="B6" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>S02</t>
         </is>
       </c>
-      <c r="D6" s="9" t="n">
+      <c r="D6" s="7" t="n">
         <v>150</v>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="E6" s="15" t="n">
         <v>0.62</v>
       </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>融合参数仅在其余五折 OOF 上拟合</t>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>融合参数仅在其余五折的折外预测（OOF）上拟合</t>
         </is>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1">
-      <c r="B7" s="8" t="n">
+      <c r="B7" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>S03</t>
         </is>
@@ -1222,41 +1945,41 @@
       <c r="D7" s="8" t="n">
         <v>150</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="14" t="n">
         <v>0.5467</v>
       </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>融合参数仅在其余五折 OOF 上拟合</t>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>融合参数仅在其余五折的折外预测（OOF）上拟合</t>
         </is>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1">
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>S04</t>
         </is>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="D8" s="7" t="n">
         <v>150</v>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="E8" s="15" t="n">
         <v>0.4867</v>
       </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>融合参数仅在其余五折 OOF 上拟合</t>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>融合参数仅在其余五折的折外预测（OOF）上拟合</t>
         </is>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1">
-      <c r="B9" s="8" t="n">
+      <c r="B9" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>S05</t>
         </is>
@@ -1264,43 +1987,43 @@
       <c r="D9" s="8" t="n">
         <v>150</v>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" s="14" t="n">
         <v>0.4867</v>
       </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>融合参数仅在其余五折 OOF 上拟合</t>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>融合参数仅在其余五折的折外预测（OOF）上拟合</t>
         </is>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1">
-      <c r="B10" s="9" t="n">
+      <c r="B10" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>S06</t>
         </is>
       </c>
-      <c r="D10" s="9" t="n">
+      <c r="D10" s="7" t="n">
         <v>150</v>
       </c>
-      <c r="E10" s="7" t="n">
+      <c r="E10" s="15" t="n">
         <v>0.5</v>
       </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>融合参数仅在其余五折 OOF 上拟合</t>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>融合参数仅在其余五折的折外预测（OOF）上拟合</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>汇总</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>S01–S06</t>
         </is>
@@ -1308,12 +2031,12 @@
       <c r="D11" s="8" t="n">
         <v>900</v>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>0.5111 ± 0.0657</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>主报表 mean±std（ddof=1）</t>
         </is>
@@ -1321,9 +2044,9 @@
     </row>
     <row r="12" ht="22" customHeight="1"/>
     <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>划分：每折 Train=750 trial / Val=150 trial；禁止随机 Val；Test=S07–S08 不参与调参。</t>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>划分：每折训练集 750 试次 / 验证集 150 试次；禁止随机验证集；测试集 S07–S08 不参与调参。</t>
         </is>
       </c>
     </row>
@@ -1341,131 +2064,130 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B2:F10"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="52" customWidth="1" min="2" max="2"/>
     <col width="25.7" customWidth="1" min="3" max="3"/>
-    <col width="45.40000000000001" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="45.4" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
     <row r="2" ht="32" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>指定集协议下的运算延迟与判定延迟</t>
+          <t>指定集实验范式下的运算延迟与判定延迟</t>
         </is>
       </c>
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="28" customHeight="1">
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>项目</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>数值</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>说明</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>状态</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>单 trial / 单窗前向（四成员融合）</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>单试次 / 单窗前向（四成员融合）</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>1.11 ms</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>RTX 5070；输入 (1,1,59,750) 同构链路实测口径</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>已实测</t>
         </is>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1">
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>采样与窗长</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>250 Hz · 750 点 = 3.00 s</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>与官方《数据说明》一致；1 trial = 1 窗</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>协议冻结</t>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>与官方《数据说明》一致；1 试次 = 1 窗</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>官方冻结</t>
         </is>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1">
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>判定延迟（指定集离线）</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>3.00 s + 1.11 ms</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>积累满 3 s trial 后给出类别；无 100 ms 滑窗 hop</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>协议上界</t>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>积累满 3 s 试次后给出类别；无 100 ms 滑窗步长</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>范式上界</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>在线系统对照（非本表主读）</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>在线系统对照（非本表主要结果）</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>判定约 3.5 s</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>仅说明同栈在线节拍；本 Excel 主读为指定集离线</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>仅说明同栈在线节拍；本 Excel 主要结果为指定集离线口径</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>附注</t>
         </is>
@@ -1473,9 +2195,9 @@
     </row>
     <row r="9" ht="22" customHeight="1"/>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>官方核心量化指标中的「运算延迟」取单 trial 前向 1.11 ms；「判定延迟」取协议窗长 3.00 s。</t>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>官方核心量化指标中的「运算延迟」取单试次前向 1.11 ms；「判定延迟」取实验范式窗长 3.00 s。</t>
         </is>
       </c>
     </row>
@@ -1493,17 +2215,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B2:H17"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="72" customWidth="1" min="2" max="2"/>
-    <col width="70.60000000000002" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="70.59999999999999" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
@@ -1516,144 +2234,144 @@
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="28" customHeight="1">
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>项目</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>数据集名称</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>主办方指定标准脑电数据集（Challenge MI）</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>数据路径</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>DATA/挑战杯运动想象赛题数据文件/</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>任务</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>3 s EEG trial → 三类：0 左手(201) / 1 右手(202) / 2 静息(204)</t>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>每试次 3 s 脑电 → 三类：0 左手(201) / 1 右手(202) / 2 静息(204)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>训练集</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>S01–S06 × 各 5 block × 30 trial = 900 trial（三类各 300）</t>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>S01–S06 × 各 5 数据块 × 30 试次 = 900 试次（三类各 300）</t>
         </is>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1">
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>测试集</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>S07–S08 × 各 2 block × 30 trial = 120 trial（无 trigger / 无标签）</t>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>S07–S08 × 各 2 数据块 × 30 试次 = 120 试次（无 trigger / 无标签）</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>采样率 / 窗</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>250 Hz；每 trial 750 点；起点 0,750,…,21750</t>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>250 Hz；每试次 750 点；起点 0,750,…,21750</t>
         </is>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1">
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>通道</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>64 信号中取 59 EEG（丢弃 ECG, HEOR, HEOL, VEOU, VEOL）；训练测试通道序一致</t>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>64 信号通道中取 59 个脑电通道（丢弃 ECG、HEOR、HEOL、VEOU、VEOL）；训练与测试通道顺序一致</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>预处理硬约束</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>先按 trial 切分，再滤波/标准化；可学习统计量仅用该折 Train 拟合</t>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>先按试次切分，再滤波/标准化；可学习统计量仅用该折训练集拟合</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>划分与主读</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>LOSO6；主读=leave-fold 嵌套 Val Acc/召/特；折内仅附报</t>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>划分与主要结果</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>留一被试交叉验证 6 折（LOSO6）；主要结果 = 逐折嵌套验证集 Acc/召/特；折内读数仅附报</t>
         </is>
       </c>
     </row>
     <row r="14" ht="38" customHeight="1">
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>交卷模型</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>QuadFold-59（59ch 从零四成员集成）；盲测 CSV 对齐 sample_submission.csv</t>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>提交模型</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>QuadFold-59（59 通道从零训练四成员集成）；盲测 CSV 与官方模板 sample_submission.csv 逐行对齐</t>
         </is>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>未使用</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>未使用测试集标签调参；本报告不含自采数据指标</t>
         </is>
@@ -1661,7 +2379,7 @@
     </row>
     <row r="16" ht="22" customHeight="1"/>
     <row r="17" ht="22" customHeight="1">
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>完整文字版见交稿包：数据集使用说明.md；官方原文副本见 原始验证数据/官方数据说明.md。</t>
         </is>
@@ -1681,12 +2399,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B2:E14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="56" customWidth="1" min="2" max="2"/>
-    <col width="39.40000000000001" customWidth="1" min="3" max="3"/>
+    <col width="39.4" customWidth="1" min="3" max="3"/>
     <col width="38.2" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
@@ -1701,153 +2419,153 @@
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="28" customHeight="1">
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>编号</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>相对路径</t>
         </is>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1">
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>D1</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>嵌套主读指标 JSON（Acc/召/特/F1/CM/六折）</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>嵌套主要结果指标 JSON（Acc/召/特/F1/混淆矩阵/六折）</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>嵌套主要结果指标 JSON（Acc/召/特/F1/混淆矩阵/六折）</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>原始验证数据/nested_N0_metrics.json</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>盲测交卷预测 CSV（官方模板已填 label）</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>盲测提交预测 CSV（官方模板已填 label）</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>原始验证数据/sample_submission.csv</t>
         </is>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1">
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>D3</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>同内容内部备份（模型名归档）</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>原始验证数据/submission_QuadFold59.csv</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>嵌套 OOF 概率 / 标签 / 被试</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>原始验证数据/oof_N0/oof_N0_*.npy</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>D5</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>官方《数据说明》副本</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>原始验证数据/官方数据说明.md</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>D6</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>本队使用对照摘录</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>原始验证数据/数据说明_使用对照.md</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>D7</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>验证过程截图 S01–S04</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>验证过程截图/</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>D8</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>交稿包（邮件附件）</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>交稿/ 或 交稿_离线验证_XH-202610.zip</t>
         </is>
@@ -1855,7 +2573,7 @@
     </row>
     <row r="13" ht="22" customHeight="1"/>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>复算嵌套指标：对 oof_N0_prob.npy 做 argmax，与 oof_N0_y.npy 对照即可复现 sheet 00/01/02。</t>
         </is>
@@ -1875,15 +2593,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:F13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B2:F14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="2" max="3"/>
     <col width="38.2" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="5" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
@@ -1896,186 +2612,192 @@
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="28" customHeight="1">
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>编号</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>文件</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>状态</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>S01</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>指定集官方数据核验：目录树、PKL 结构（data 64×22500、ch_names、srate=250）、train 900 / test 120 计数（终端回放）</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>验证过程截图/S01_数据集结构与加载核验.png</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>S02</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>嵌套 N0 主读回放运行：replay_nested.py 现场输出六折 Acc 与 0.511±0.066（终端回放）</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>嵌套验证主结果回放运行：replay_nested.py 现场输出六折 Acc 与 0.511±0.066（终端回放）</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>验证过程截图/S02_嵌套N0指标汇总.png</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>S03</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>盲测交卷 CSV 再生成与比对：predict_submission.py 现场重生成，与交稿 CSV 逐行 diff（终端回放）</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>验证过程截图/S03_交卷CSV再生成与比对.png</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>盲测提交 CSV 再生成与比对：predict_submission.py 现场重生成，与提交 CSV 逐行比对（终端回放）</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>验证过程截图/S03_提交CSV再生成与比对.png</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>S04</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>指定集指标独立复算：从 OOF npy 重算 Acc/召/特/F1/CM/六折，逐项对照登记 JSON（终端回放）</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>验证过程截图/S04_独立复算.png</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>S05</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>交卷 CSV 完整性：120 行、表头一致、sample_id 与官方模板逐行对齐、取值合法（终端回放）</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>验证过程截图/S05_交卷CSV完整性校验.png</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>提交 CSV 完整性：120 行、表头一致、sample_id 与官方模板逐行对齐、取值合法（终端回放）</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>验证过程截图/S05_提交CSV完整性校验.png</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>S06</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>Excel 核心指标与登记 JSON 一致性：程序化读取 00 表单元格对照（终端回放）</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>验证过程截图/S06_Excel与JSON一致性.png</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>S07</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>交稿包文件 MD5 指纹与运行环境（python/numpy 版本、时间戳；终端回放）</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>验证过程截图/S07_文件指纹与环境.png</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13">
-      <c r="B13" s="2" t="inlineStr">
+    <row r="13" ht="15" customHeight="1">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>下列嵌入图便于审阅；原图亦在交稿包 验证过程截图/ 目录。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>注：S07 中 xlsx 自身 MD5 为嵌入本截图前一版的指纹（自引用无法自洽）；交稿包核验以 S07 其余 13 项文件指纹为准。</t>
         </is>
       </c>
     </row>
@@ -2094,95 +2816,93 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B2:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="15.6" customWidth="1" min="2" max="2"/>
-    <col width="63.60000000000002" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="63.6" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
     <row r="2" ht="32" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>交卷决策与评测纪律（指定集）</t>
+          <t>提交决策与评测纪律（指定集）</t>
         </is>
       </c>
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="28" customHeight="1">
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>项</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>说明</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>交卷模型</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>QuadFold-59（嵌套主读 0.511±0.066）</t>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>提交模型</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>QuadFold-59（嵌套主要结果 0.5111 ± 0.0657）</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>主读尺子</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>LOSO6 leave-fold 嵌套；禁止用折内 0.558 作对外主读</t>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>主要结果口径</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>留一被试交叉验证 6 折嵌套；折内 0.5580 仅内部参考，不作为对外报告结果</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>盲测文件</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>sample_submission.csv（官方模板已填 label∈{0,1,2}，120 行）</t>
         </is>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1">
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>风险否决（归档）</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>备选 8ch 微调栈嵌套 0.540：test 预测 Rest≈51% 落在 Val 支撑外，不交</t>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>备选 8 通道微调方案嵌套 0.540：测试集预测静息类占比约 51%，超出验证集支撑范围，不提交</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>纪律</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>超参与融合权仅在 Val/嵌套折外选定；测试标签未用于调参</t>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>超参数与融合权重仅在验证集/嵌套折外选定；测试集标签未用于调参</t>
         </is>
       </c>
     </row>
@@ -2200,15 +2920,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:F12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B2:F12"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="3" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
@@ -2221,145 +2938,145 @@
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="28" customHeight="1">
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>核对项</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>期望</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>表内</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>状态</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>准确率</t>
         </is>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="14" t="n">
         <v>0.5111</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" s="14" t="n">
         <v>0.5111</v>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>召回率 macro</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="15" t="n">
         <v>0.5111</v>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="15" t="n">
         <v>0.5111</v>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>特异性 macro</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="14" t="n">
         <v>0.7556</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="14" t="n">
         <v>0.7556</v>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>运算延迟</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>1.11 ms</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>1.11 ms</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>判定延迟（指定集）</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>3.00 s</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>3.00 s</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>OOF 试次数</t>
         </is>
       </c>
-      <c r="C10" s="9" t="n">
+      <c r="C10" s="7" t="n">
         <v>900</v>
       </c>
-      <c r="D10" s="9" t="n">
+      <c r="D10" s="7" t="n">
         <v>900</v>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>盲测 CSV 行数</t>
         </is>
@@ -2370,29 +3087,29 @@
       <c r="D11" s="8" t="n">
         <v>120</v>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>本报告是否含自采指标</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>

</xml_diff>